<commit_message>
Oprav připomínky z ostrého provozu
</commit_message>
<xml_diff>
--- a/Sklad_new.xlsx
+++ b/Sklad_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lukasseifert/Vibecoding/Cater_sklad/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{897AB730-06D3-EC4F-BA32-BB9568A3EDC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6944C2F-1701-4740-B146-EF3334F75754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="21560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="780" windowWidth="36000" windowHeight="21560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="List 1 - Sešit4" sheetId="1" r:id="rId1"/>

</xml_diff>